<commit_message>
Infer date validation for date/time columns
Date/time columns now auto-enforce date-ness the same way numeric
columns auto-enforce ISNUMBER: a DateTime/DateTimeOffset/DateOnly/TimeOnly
column with no explicit Range gets a date validation across Excel's full
supported span [1900-01-01, 9999-12-31], so manually-typed text is
blocked while any real date is accepted.
Adds IsTemporalType(), an IsDate flag on ColumnConfig mirroring IsNumber,
and HasDateValidation. Like the numeric ISNUMBER check, this is always on,
independent of inferValidationFromTypes.
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/ColumnWidths.FontMatrix.verified.xlsx
+++ b/src/Excelsior.Tests/ColumnWidths.FontMatrix.verified.xlsx
@@ -243,11 +243,13 @@
     <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a number." prompt="Required field" sqref="C2:C3">
       <formula1>ISNUMBER(C2)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." prompt="Required field" sqref="D2:D3">
-      <formula1>LEN(TRIM(D2))&gt;0</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." prompt="Required field" sqref="E2:E3">
-      <formula1>LEN(TRIM(E2))&gt;0</formula1>
+    <dataValidation type="date" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date." prompt="Required field" sqref="D2:D3">
+      <formula1>2</formula1>
+      <formula2>2958465</formula2>
+    </dataValidation>
+    <dataValidation type="date" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date." prompt="Required field" sqref="E2:E3">
+      <formula1>2</formula1>
+      <formula2>2958465</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: TRUE, FALSE." prompt="Select one of: TRUE, FALSE" sqref="F2:F3">
       <formula1>"TRUE,FALSE"</formula1>

</xml_diff>

<commit_message>
Infer date validation for date/time columns (#235)
Date/time columns now auto-enforce date-ness the same way numeric
columns auto-enforce ISNUMBER: a DateTime/DateTimeOffset/DateOnly/TimeOnly
column with no explicit Range gets a date validation across Excel's full
supported span [1900-01-01, 9999-12-31], so manually-typed text is
blocked while any real date is accepted.
Adds IsTemporalType(), an IsDate flag on ColumnConfig mirroring IsNumber,
and HasDateValidation. Like the numeric ISNUMBER check, this is always on,
independent of inferValidationFromTypes.
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/ColumnWidths.FontMatrix.verified.xlsx
+++ b/src/Excelsior.Tests/ColumnWidths.FontMatrix.verified.xlsx
@@ -243,11 +243,13 @@
     <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a number." prompt="Required field" sqref="C2:C3">
       <formula1>ISNUMBER(C2)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." prompt="Required field" sqref="D2:D3">
-      <formula1>LEN(TRIM(D2))&gt;0</formula1>
-    </dataValidation>
-    <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="This field is required." prompt="Required field" sqref="E2:E3">
-      <formula1>LEN(TRIM(E2))&gt;0</formula1>
+    <dataValidation type="date" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date." prompt="Required field" sqref="D2:D3">
+      <formula1>2</formula1>
+      <formula2>2958465</formula2>
+    </dataValidation>
+    <dataValidation type="date" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date." prompt="Required field" sqref="E2:E3">
+      <formula1>2</formula1>
+      <formula2>2958465</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be one of: TRUE, FALSE." prompt="Select one of: TRUE, FALSE" sqref="F2:F3">
       <formula1>"TRUE,FALSE"</formula1>

</xml_diff>

<commit_message>
Word date validation message by temporal kind, with format (#236)
* Word date-validation message by temporal kind, with format

* .

* .
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/ColumnWidths.FontMatrix.verified.xlsx
+++ b/src/Excelsior.Tests/ColumnWidths.FontMatrix.verified.xlsx
@@ -243,11 +243,11 @@
     <dataValidation type="custom" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a number." prompt="Required field" sqref="C2:C3">
       <formula1>ISNUMBER(C2)</formula1>
     </dataValidation>
-    <dataValidation type="date" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date." prompt="Required field" sqref="D2:D3">
+    <dataValidation type="date" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date and time.&#10;yyyy-MM-dd HH:mm:ss" prompt="Date and time as yyyy-MM-dd HH:mm:ss" sqref="D2:D3">
       <formula1>2</formula1>
       <formula2>2958465</formula2>
     </dataValidation>
-    <dataValidation type="date" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date." prompt="Required field" sqref="E2:E3">
+    <dataValidation type="date" operator="between" allowBlank="0" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid value" error="Must be a valid date.&#10;yyyy-MM-dd" prompt="Date as yyyy-MM-dd" sqref="E2:E3">
       <formula1>2</formula1>
       <formula2>2958465</formula2>
     </dataValidation>

</xml_diff>